<commit_message>
fix: Excel export sheet-name collisions, timing, and column labels
- Sheet names now dedup after the 31-character truncation instead of
  silently colliding and overwriting an earlier strategy's data.
- The Markov QALY sheet's Time (yrs) column used the interval start while
  its own Discount Factor column used the interval midpoint; use the same
  interval_times for both.
- export_excel_model's PH/AFT wrappers resolve the baseline before writing
  the hazard-ratio/acceleration-factor cell, so an unsupported baseline no
  longer leaves an editable input that nothing references.
- Renamed export_excel_model's (raw) columns to (occ): they hold the
  half-cycle-corrected occupancy-weighted reward, which is what
  export_to_excel calls (HCC), not what it calls (raw).
</commit_message>
<xml_diff>
--- a/examples/psm_oncology/workbooks/base_case.xlsx
+++ b/examples/psm_oncology/workbooks/base_case.xlsx
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M28" s="3" t="inlineStr">
         <is>
-          <t>drug(raw)</t>
+          <t>drug(occ)</t>
         </is>
       </c>
       <c r="N28" s="3" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>prog_care(raw)</t>
+          <t>prog_care(occ)</t>
         </is>
       </c>
       <c r="P28" s="3" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="Q28" s="3" t="inlineStr">
         <is>
-          <t>bsc(raw)</t>
+          <t>bsc(occ)</t>
         </is>
       </c>
       <c r="R28" s="3" t="inlineStr">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="S28" s="3" t="inlineStr">
         <is>
-          <t>ae(raw)</t>
+          <t>ae(occ)</t>
         </is>
       </c>
       <c r="T28" s="3" t="inlineStr">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="V28" s="3" t="inlineStr">
         <is>
-          <t>QALY(raw)</t>
+          <t>QALY(occ)</t>
         </is>
       </c>
       <c r="W28" s="3" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="X28" s="3" t="inlineStr">
         <is>
-          <t>LY(raw)</t>
+          <t>LY(occ)</t>
         </is>
       </c>
       <c r="Y28" s="3" t="inlineStr">
@@ -26008,7 +26008,7 @@
       </c>
       <c r="M28" s="3" t="inlineStr">
         <is>
-          <t>drug(raw)</t>
+          <t>drug(occ)</t>
         </is>
       </c>
       <c r="N28" s="3" t="inlineStr">
@@ -26018,7 +26018,7 @@
       </c>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>prog_care(raw)</t>
+          <t>prog_care(occ)</t>
         </is>
       </c>
       <c r="P28" s="3" t="inlineStr">
@@ -26028,7 +26028,7 @@
       </c>
       <c r="Q28" s="3" t="inlineStr">
         <is>
-          <t>bsc(raw)</t>
+          <t>bsc(occ)</t>
         </is>
       </c>
       <c r="R28" s="3" t="inlineStr">
@@ -26038,7 +26038,7 @@
       </c>
       <c r="S28" s="3" t="inlineStr">
         <is>
-          <t>ae(raw)</t>
+          <t>ae(occ)</t>
         </is>
       </c>
       <c r="T28" s="3" t="inlineStr">
@@ -26053,7 +26053,7 @@
       </c>
       <c r="V28" s="3" t="inlineStr">
         <is>
-          <t>QALY(raw)</t>
+          <t>QALY(occ)</t>
         </is>
       </c>
       <c r="W28" s="3" t="inlineStr">
@@ -26063,7 +26063,7 @@
       </c>
       <c r="X28" s="3" t="inlineStr">
         <is>
-          <t>LY(raw)</t>
+          <t>LY(occ)</t>
         </is>
       </c>
       <c r="Y28" s="3" t="inlineStr">

</xml_diff>